<commit_message>
Update 周四 2026/08/06 12:02:18
</commit_message>
<xml_diff>
--- a/模板库/标准库模板.xlsx
+++ b/模板库/标准库模板.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17680"/>
+    <workbookView windowWidth="20400" windowHeight="11480"/>
   </bookViews>
   <sheets>
     <sheet name="标准条件" sheetId="1" r:id="rId1"/>
@@ -133,7 +133,7 @@
     <t>振动测试</t>
   </si>
   <si>
-    <t>比亚迪</t>
+    <t>洛科</t>
   </si>
   <si>
     <t>BYD-Q-SC 001 5.2</t>
@@ -145,7 +145,7 @@
     <t>功能等级A。</t>
   </si>
   <si>
-    <t>蔚来</t>
+    <t>捷途</t>
   </si>
   <si>
     <t>NIO-TS-018 6.1</t>
@@ -218,7 +218,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,13 +245,6 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF808080"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -730,148 +723,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>